<commit_message>
Figure updates + added mappings.json
</commit_message>
<xml_diff>
--- a/Research/Workflow Analysis/Workflow_Analysis.xlsx
+++ b/Research/Workflow Analysis/Workflow_Analysis.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10525"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marci/Downloads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/marci/Desktop/Creative-Visual-Design-Accessibility-Tools/Research/Workflow Analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02DD1C54-8B1E-6D41-A8B9-9B5DC6F95A17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2A5392E-C85A-D749-B612-83585A8546D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-20" yWindow="760" windowWidth="29400" windowHeight="17340" firstSheet="3" activeTab="12" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17340" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="TEMPLATE" sheetId="1" r:id="rId1"/>
@@ -443,11 +443,6 @@
     <t>the hardest part of this action is that it is multistep and requires scrolling which is frustrating with voice</t>
   </si>
   <si>
-    <t xml:space="preserve">
-ASMR UI Designing in FIGMA - STRIPE - No Talking | Silent
-ASMR UI Designing in FIGMA - STRIPE - No Talking | Silent</t>
-  </si>
-  <si>
     <t>https://www.youtube.com/watch?v=OLb7Rqo1KVQ</t>
   </si>
   <si>
@@ -1115,6 +1110,9 @@
   </si>
   <si>
     <t>[hover] over [reference(s)] on [canvas]</t>
+  </si>
+  <si>
+    <t>ASMR UI Designing in FIGMA - STRIPE - No Talking | Silent</t>
   </si>
 </sst>
 </file>
@@ -6683,11 +6681,11 @@
         <v>0</v>
       </c>
       <c r="Q194">
-        <f t="shared" ref="Q194:Q225" si="38">P194-O194</f>
+        <f t="shared" ref="Q194:Q200" si="38">P194-O194</f>
         <v>0</v>
       </c>
       <c r="R194" t="str">
-        <f t="shared" ref="R194:R225" si="39">IF(Q194=0,"&lt;1 second","&lt;"&amp;(ROUND(Q194,2)+1)&amp;" seconds")</f>
+        <f t="shared" ref="R194:R200" si="39">IF(Q194=0,"&lt;1 second","&lt;"&amp;(ROUND(Q194,2)+1)&amp;" seconds")</f>
         <v>&lt;1 second</v>
       </c>
       <c r="S194">
@@ -6968,13 +6966,13 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>331</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>332</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" t="s">
         <v>333</v>
-      </c>
-      <c r="C2" t="s">
-        <v>334</v>
       </c>
       <c r="D2" s="3">
         <v>55.48</v>
@@ -6983,7 +6981,7 @@
         <v>55.54</v>
       </c>
       <c r="F2" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="G2" t="s">
         <v>85</v>
@@ -7322,13 +7320,13 @@
         <v>56.05</v>
       </c>
       <c r="G9" t="s">
+        <v>226</v>
+      </c>
+      <c r="I9" t="s">
         <v>227</v>
       </c>
-      <c r="I9" t="s">
-        <v>228</v>
-      </c>
       <c r="J9" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="K9" t="s">
         <v>43</v>
@@ -7465,7 +7463,7 @@
         <v>56.2</v>
       </c>
       <c r="F12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="G12" t="s">
         <v>99</v>
@@ -7611,7 +7609,7 @@
         <v>56.29</v>
       </c>
       <c r="F15" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="G15" t="s">
         <v>85</v>
@@ -7757,7 +7755,7 @@
         <v>56.35</v>
       </c>
       <c r="F18" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G18" t="s">
         <v>45</v>
@@ -7807,7 +7805,7 @@
         <v>56.38</v>
       </c>
       <c r="F19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="G19" t="s">
         <v>50</v>
@@ -7858,7 +7856,7 @@
         <v>56.39</v>
       </c>
       <c r="G20" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I20" t="s">
         <v>29</v>
@@ -7952,7 +7950,7 @@
         <v>56.48</v>
       </c>
       <c r="G22" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I22" t="s">
         <v>29</v>
@@ -8306,13 +8304,13 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>338</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>339</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" t="s">
         <v>340</v>
-      </c>
-      <c r="C2" t="s">
-        <v>341</v>
       </c>
       <c r="D2" s="3">
         <v>57</v>
@@ -8321,13 +8319,13 @@
         <v>57.02</v>
       </c>
       <c r="G2" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I2" t="s">
         <v>46</v>
       </c>
       <c r="J2" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K2" t="s">
         <v>92</v>
@@ -8371,13 +8369,13 @@
         <v>57.03</v>
       </c>
       <c r="G3" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I3" t="s">
         <v>46</v>
       </c>
       <c r="J3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K3" t="s">
         <v>92</v>
@@ -8472,7 +8470,7 @@
         <v>57.06</v>
       </c>
       <c r="F5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="G5" t="s">
         <v>32</v>
@@ -8522,7 +8520,7 @@
         <v>57.1</v>
       </c>
       <c r="F6" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="G6" t="s">
         <v>32</v>
@@ -8572,16 +8570,16 @@
         <v>57.11</v>
       </c>
       <c r="F7" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="G7" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I7" t="s">
         <v>77</v>
       </c>
       <c r="J7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K7" t="s">
         <v>92</v>
@@ -8622,7 +8620,7 @@
         <v>57.12</v>
       </c>
       <c r="G8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I8" t="s">
         <v>29</v>
@@ -8718,13 +8716,13 @@
         <v>57.13</v>
       </c>
       <c r="G10" t="s">
+        <v>226</v>
+      </c>
+      <c r="I10" t="s">
         <v>227</v>
       </c>
-      <c r="I10" t="s">
-        <v>228</v>
-      </c>
       <c r="J10" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="K10" t="s">
         <v>43</v>
@@ -8813,7 +8811,7 @@
         <v>57.17</v>
       </c>
       <c r="F12" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="G12" t="s">
         <v>82</v>
@@ -8863,7 +8861,7 @@
         <v>57.2</v>
       </c>
       <c r="F13" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="G13" t="s">
         <v>32</v>
@@ -8913,13 +8911,13 @@
         <v>57.22</v>
       </c>
       <c r="G14" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I14" t="s">
         <v>46</v>
       </c>
       <c r="J14" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K14" t="s">
         <v>92</v>
@@ -9058,7 +9056,7 @@
         <v>57.26</v>
       </c>
       <c r="F17" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="G17" t="s">
         <v>45</v>
@@ -9108,7 +9106,7 @@
         <v>57.47</v>
       </c>
       <c r="F18" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="G18" t="s">
         <v>32</v>
@@ -9159,7 +9157,7 @@
         <v>57.51</v>
       </c>
       <c r="G19" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I19" t="s">
         <v>29</v>
@@ -9255,7 +9253,7 @@
         <v>57.51</v>
       </c>
       <c r="G21" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="I21" t="s">
         <v>74</v>
@@ -9302,7 +9300,7 @@
         <v>57.56</v>
       </c>
       <c r="F22" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="G22" t="s">
         <v>32</v>
@@ -9353,7 +9351,7 @@
         <v>57.57</v>
       </c>
       <c r="G23" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I23" t="s">
         <v>29</v>
@@ -9449,7 +9447,7 @@
         <v>58.02</v>
       </c>
       <c r="G25" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I25" t="s">
         <v>74</v>
@@ -9760,7 +9758,7 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="B1" t="s">
         <v>8</v>
@@ -9807,10 +9805,10 @@
         <v>95</v>
       </c>
       <c r="B5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.2">
@@ -9832,7 +9830,7 @@
         <v>100</v>
       </c>
       <c r="C7" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.2">
@@ -9854,7 +9852,7 @@
         <v>101</v>
       </c>
       <c r="C9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.2">
@@ -9876,7 +9874,7 @@
         <v>54</v>
       </c>
       <c r="C11" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.2">
@@ -9887,7 +9885,7 @@
         <v>74</v>
       </c>
       <c r="C12" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.2">
@@ -9906,7 +9904,7 @@
         <v>117</v>
       </c>
       <c r="B14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="C14" t="s">
         <v>97</v>
@@ -9914,13 +9912,13 @@
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B15" t="s">
         <v>78</v>
       </c>
       <c r="C15" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.2">
@@ -9928,10 +9926,10 @@
         <v>120</v>
       </c>
       <c r="B16" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="C16" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.2">
@@ -9939,7 +9937,7 @@
         <v>24</v>
       </c>
       <c r="B17" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="C17" t="s">
         <v>25</v>
@@ -9958,21 +9956,21 @@
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="B19" t="s">
         <v>97</v>
       </c>
       <c r="C19" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B20" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C20" t="s">
         <v>74</v>
@@ -9980,10 +9978,10 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B21" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C21" t="s">
         <v>112</v>
@@ -9991,7 +9989,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B22" t="s">
         <v>96</v>
@@ -10002,7 +10000,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B23" t="s">
         <v>77</v>
@@ -10013,7 +10011,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B24" t="s">
         <v>115</v>
@@ -10030,18 +10028,18 @@
         <v>57</v>
       </c>
       <c r="C25" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B26" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="C26" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.2">
@@ -10049,7 +10047,7 @@
         <v>64</v>
       </c>
       <c r="B27" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="C27" t="s">
         <v>42</v>
@@ -10057,18 +10055,18 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B28" t="s">
         <v>81</v>
       </c>
       <c r="C28" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B29" t="s">
         <v>42</v>
@@ -10079,7 +10077,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="B30" t="s">
         <v>29</v>
@@ -10093,7 +10091,7 @@
         <v>50</v>
       </c>
       <c r="B31" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C31" t="s">
         <v>101</v>
@@ -10112,7 +10110,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="C33" t="s">
         <v>52</v>
@@ -10120,7 +10118,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="C34" t="s">
         <v>72</v>
@@ -10128,7 +10126,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="C35" t="s">
         <v>26</v>
@@ -10136,15 +10134,15 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="C36" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C37" t="s">
         <v>84</v>
@@ -10152,15 +10150,15 @@
     </row>
     <row r="38" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C38" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="C39" t="s">
         <v>126</v>
@@ -10168,7 +10166,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="C40" t="s">
         <v>118</v>
@@ -10176,7 +10174,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C41" t="s">
         <v>111</v>
@@ -10184,31 +10182,31 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="C42" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C43" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="C44" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C45" t="s">
         <v>59</v>
@@ -10216,17 +10214,17 @@
     </row>
     <row r="46" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="47" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="48" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.2">
@@ -10246,32 +10244,32 @@
     </row>
     <row r="52" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="53" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
     </row>
     <row r="54" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
     </row>
     <row r="55" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
     </row>
     <row r="56" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
     </row>
     <row r="57" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
     </row>
     <row r="58" spans="1:1" x14ac:dyDescent="0.2">
@@ -10291,7 +10289,7 @@
     </row>
     <row r="61" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
@@ -12269,11 +12267,11 @@
         <v>40</v>
       </c>
       <c r="Q34">
-        <f t="shared" ref="Q34:Q65" si="8">P34-O34</f>
+        <f t="shared" ref="Q34:Q52" si="8">P34-O34</f>
         <v>0</v>
       </c>
       <c r="R34" t="str">
-        <f t="shared" ref="R34:R65" si="9">IF(Q34=0,"&lt;1 second","&lt;"&amp;(ROUND(Q34,2)+1)&amp;" seconds")</f>
+        <f t="shared" ref="R34:R52" si="9">IF(Q34=0,"&lt;1 second","&lt;"&amp;(ROUND(Q34,2)+1)&amp;" seconds")</f>
         <v>&lt;1 second</v>
       </c>
       <c r="S34" s="3">
@@ -13734,13 +13732,13 @@
     </row>
     <row r="2" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="12" t="s">
+        <v>355</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" t="s">
         <v>133</v>
-      </c>
-      <c r="C2" t="s">
-        <v>134</v>
       </c>
       <c r="D2" s="3">
         <v>0.1</v>
@@ -13749,7 +13747,7 @@
         <v>0.13</v>
       </c>
       <c r="F2" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G2" t="s">
         <v>45</v>
@@ -13802,7 +13800,7 @@
         <v>0.14000000000000001</v>
       </c>
       <c r="F3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="G3" s="11" t="s">
         <v>32</v>
@@ -13855,7 +13853,7 @@
         <v>0.15</v>
       </c>
       <c r="F4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G4" s="11" t="s">
         <v>32</v>
@@ -13873,7 +13871,7 @@
         <v>35</v>
       </c>
       <c r="N4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="O4">
         <f t="shared" si="0"/>
@@ -13908,7 +13906,7 @@
         <v>0.2</v>
       </c>
       <c r="F5" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="G5" s="11" t="s">
         <v>32</v>
@@ -13926,7 +13924,7 @@
         <v>35</v>
       </c>
       <c r="N5" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="O5">
         <f t="shared" si="0"/>
@@ -13961,7 +13959,7 @@
         <v>0.23</v>
       </c>
       <c r="F6" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="G6" t="s">
         <v>56</v>
@@ -13979,7 +13977,7 @@
         <v>28</v>
       </c>
       <c r="N6" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="O6">
         <f t="shared" si="0"/>
@@ -14014,16 +14012,16 @@
         <v>0.26</v>
       </c>
       <c r="F7" t="s">
+        <v>142</v>
+      </c>
+      <c r="G7" s="14" t="s">
         <v>143</v>
-      </c>
-      <c r="G7" s="14" t="s">
-        <v>144</v>
       </c>
       <c r="I7" t="s">
         <v>77</v>
       </c>
       <c r="J7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K7" t="s">
         <v>27</v>
@@ -14032,7 +14030,7 @@
         <v>28</v>
       </c>
       <c r="N7" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="O7">
         <f t="shared" si="0"/>
@@ -14067,16 +14065,16 @@
         <v>0.28999999999999998</v>
       </c>
       <c r="F8" t="s">
+        <v>146</v>
+      </c>
+      <c r="G8" s="14" t="s">
         <v>147</v>
-      </c>
-      <c r="G8" s="14" t="s">
-        <v>148</v>
       </c>
       <c r="I8" t="s">
         <v>83</v>
       </c>
       <c r="J8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K8" t="s">
         <v>27</v>
@@ -14085,7 +14083,7 @@
         <v>28</v>
       </c>
       <c r="N8" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O8">
         <f t="shared" si="0"/>
@@ -14120,16 +14118,16 @@
         <v>0.31</v>
       </c>
       <c r="F9" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I9" t="s">
         <v>83</v>
       </c>
       <c r="J9" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K9" t="s">
         <v>27</v>
@@ -14138,7 +14136,7 @@
         <v>28</v>
       </c>
       <c r="N9" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O9">
         <f t="shared" si="0"/>
@@ -14211,16 +14209,16 @@
         <v>0.39</v>
       </c>
       <c r="F11" t="s">
+        <v>151</v>
+      </c>
+      <c r="G11" s="14" t="s">
         <v>152</v>
       </c>
-      <c r="G11" s="14" t="s">
+      <c r="I11" t="s">
         <v>153</v>
       </c>
-      <c r="I11" t="s">
-        <v>154</v>
-      </c>
       <c r="J11" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K11" t="s">
         <v>27</v>
@@ -14229,7 +14227,7 @@
         <v>28</v>
       </c>
       <c r="N11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="O11">
         <f t="shared" si="0"/>
@@ -14264,16 +14262,16 @@
         <v>0.46</v>
       </c>
       <c r="F12" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="G12" s="14" t="s">
+        <v>152</v>
+      </c>
+      <c r="I12" t="s">
         <v>153</v>
       </c>
-      <c r="I12" t="s">
-        <v>154</v>
-      </c>
       <c r="J12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="K12" t="s">
         <v>27</v>
@@ -14282,7 +14280,7 @@
         <v>28</v>
       </c>
       <c r="N12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="O12">
         <f t="shared" si="0"/>
@@ -14318,16 +14316,16 @@
         <v>0.47</v>
       </c>
       <c r="F13" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="G13" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I13" t="s">
         <v>77</v>
       </c>
       <c r="J13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K13" t="s">
         <v>27</v>
@@ -14336,7 +14334,7 @@
         <v>28</v>
       </c>
       <c r="N13" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="O13">
         <f t="shared" si="0"/>
@@ -14371,16 +14369,16 @@
         <v>0.5</v>
       </c>
       <c r="F14" t="s">
+        <v>158</v>
+      </c>
+      <c r="G14" s="14" t="s">
         <v>159</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>160</v>
       </c>
       <c r="I14" t="s">
         <v>46</v>
       </c>
       <c r="J14" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K14" t="s">
         <v>92</v>
@@ -14425,16 +14423,16 @@
         <v>0.51</v>
       </c>
       <c r="F15" t="s">
+        <v>161</v>
+      </c>
+      <c r="G15" t="s">
         <v>162</v>
-      </c>
-      <c r="G15" t="s">
-        <v>163</v>
       </c>
       <c r="I15" t="s">
         <v>46</v>
       </c>
       <c r="J15" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K15" t="s">
         <v>92</v>
@@ -14478,16 +14476,16 @@
         <v>0.54</v>
       </c>
       <c r="F16" t="s">
+        <v>164</v>
+      </c>
+      <c r="G16" s="14" t="s">
         <v>165</v>
-      </c>
-      <c r="G16" s="14" t="s">
-        <v>166</v>
       </c>
       <c r="I16" t="s">
         <v>46</v>
       </c>
       <c r="J16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K16" t="s">
         <v>92</v>
@@ -14532,7 +14530,7 @@
         <v>0.55000000000000004</v>
       </c>
       <c r="F17" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="G17" s="14" t="s">
         <v>41</v>
@@ -14585,16 +14583,16 @@
         <v>0.56000000000000005</v>
       </c>
       <c r="F18" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="G18" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I18" t="s">
         <v>46</v>
       </c>
       <c r="J18" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K18" t="s">
         <v>92</v>
@@ -14639,7 +14637,7 @@
         <v>0.57999999999999996</v>
       </c>
       <c r="F19" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="G19" s="11" t="s">
         <v>32</v>
@@ -14693,7 +14691,7 @@
         <v>0.59</v>
       </c>
       <c r="F20" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="G20" t="s">
         <v>45</v>
@@ -14746,16 +14744,16 @@
         <v>1.01</v>
       </c>
       <c r="F21" t="s">
+        <v>170</v>
+      </c>
+      <c r="G21" s="14" t="s">
         <v>171</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>172</v>
       </c>
       <c r="I21" t="s">
         <v>57</v>
       </c>
       <c r="J21" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K21" t="s">
         <v>27</v>
@@ -14764,7 +14762,7 @@
         <v>28</v>
       </c>
       <c r="N21" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="O21">
         <f t="shared" si="0"/>
@@ -14800,16 +14798,16 @@
         <v>1.02</v>
       </c>
       <c r="F22" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G22" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I22" t="s">
         <v>46</v>
       </c>
       <c r="J22" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K22" t="s">
         <v>92</v>
@@ -14854,16 +14852,16 @@
         <v>1.03</v>
       </c>
       <c r="F23" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="G23" s="14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I23" t="s">
         <v>83</v>
       </c>
       <c r="J23" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K23" t="s">
         <v>27</v>
@@ -14872,7 +14870,7 @@
         <v>28</v>
       </c>
       <c r="N23" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O23">
         <f t="shared" si="0"/>
@@ -14908,7 +14906,7 @@
         <v>1.05</v>
       </c>
       <c r="F24" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="G24" t="s">
         <v>51</v>
@@ -14961,16 +14959,16 @@
         <v>1.0900000000000001</v>
       </c>
       <c r="F25" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="G25" s="14" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I25" t="s">
         <v>83</v>
       </c>
       <c r="J25" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K25" t="s">
         <v>27</v>
@@ -14979,7 +14977,7 @@
         <v>28</v>
       </c>
       <c r="N25" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="O25">
         <f t="shared" si="0"/>
@@ -15015,7 +15013,7 @@
         <v>1.1200000000000001</v>
       </c>
       <c r="F26" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="G26" t="s">
         <v>24</v>
@@ -15033,7 +15031,7 @@
         <v>28</v>
       </c>
       <c r="N26" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="O26">
         <f t="shared" si="0"/>
@@ -15284,13 +15282,13 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>181</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" t="s">
         <v>182</v>
-      </c>
-      <c r="C2" t="s">
-        <v>183</v>
       </c>
       <c r="D2" s="3">
         <v>10.36</v>
@@ -15402,13 +15400,13 @@
         <v>10.37</v>
       </c>
       <c r="G4" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I4" s="15" t="s">
         <v>81</v>
       </c>
       <c r="J4" s="15" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K4" t="s">
         <v>43</v>
@@ -15417,7 +15415,7 @@
         <v>28</v>
       </c>
       <c r="N4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="O4">
         <f t="shared" si="0"/>
@@ -15504,7 +15502,7 @@
         <v>10.38</v>
       </c>
       <c r="G6" s="14" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="I6" t="s">
         <v>29</v>
@@ -15554,16 +15552,16 @@
         <v>10.4</v>
       </c>
       <c r="F7" t="s">
+        <v>187</v>
+      </c>
+      <c r="G7" s="14" t="s">
         <v>188</v>
       </c>
-      <c r="G7" s="14" t="s">
+      <c r="I7" t="s">
         <v>189</v>
       </c>
-      <c r="I7" t="s">
-        <v>190</v>
-      </c>
       <c r="J7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="K7" t="s">
         <v>119</v>
@@ -15572,7 +15570,7 @@
         <v>66</v>
       </c>
       <c r="N7" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="O7">
         <f t="shared" si="0"/>
@@ -15659,10 +15657,10 @@
         <v>10.41</v>
       </c>
       <c r="F9" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="G9" s="14" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I9" t="s">
         <v>29</v>
@@ -15863,13 +15861,13 @@
         <v>10.46</v>
       </c>
       <c r="G13" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I13" t="s">
         <v>46</v>
       </c>
       <c r="J13" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K13" t="s">
         <v>92</v>
@@ -15928,7 +15926,7 @@
         <v>35</v>
       </c>
       <c r="N14" s="15" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="O14">
         <f t="shared" si="0"/>
@@ -15963,13 +15961,13 @@
         <v>10.52</v>
       </c>
       <c r="G15" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I15" t="s">
         <v>46</v>
       </c>
       <c r="J15" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K15" t="s">
         <v>92</v>
@@ -16014,13 +16012,13 @@
         <v>10.52</v>
       </c>
       <c r="G16" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I16" t="s">
         <v>46</v>
       </c>
       <c r="J16" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K16" t="s">
         <v>92</v>
@@ -16065,13 +16063,13 @@
         <v>10.53</v>
       </c>
       <c r="G17" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I17" t="s">
         <v>46</v>
       </c>
       <c r="J17" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K17" t="s">
         <v>92</v>
@@ -16166,13 +16164,13 @@
         <v>10.55</v>
       </c>
       <c r="G19" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I19" t="s">
         <v>46</v>
       </c>
       <c r="J19" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K19" t="s">
         <v>92</v>
@@ -16217,13 +16215,13 @@
         <v>10.57</v>
       </c>
       <c r="G20" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I20" t="s">
         <v>46</v>
       </c>
       <c r="J20" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K20" t="s">
         <v>92</v>
@@ -16283,7 +16281,7 @@
         <v>28</v>
       </c>
       <c r="N21" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="O21">
         <f t="shared" si="0"/>
@@ -16369,16 +16367,16 @@
         <v>10.59</v>
       </c>
       <c r="F23" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="G23" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I23" t="s">
         <v>77</v>
       </c>
       <c r="J23" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K23" t="s">
         <v>27</v>
@@ -16473,13 +16471,13 @@
         <v>11</v>
       </c>
       <c r="G25" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I25" t="s">
         <v>46</v>
       </c>
       <c r="J25" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K25" t="s">
         <v>92</v>
@@ -16523,13 +16521,13 @@
         <v>11.03</v>
       </c>
       <c r="G26" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I26" t="s">
         <v>46</v>
       </c>
       <c r="J26" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K26" t="s">
         <v>92</v>
@@ -16933,13 +16931,13 @@
         <v>11.08</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I34" t="s">
         <v>81</v>
       </c>
       <c r="J34" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K34" t="s">
         <v>43</v>
@@ -16948,7 +16946,7 @@
         <v>28</v>
       </c>
       <c r="N34" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="O34">
         <f t="shared" ref="O34:O67" si="7">(INT(D34)*60+(D34-INT(D34))*100)-(INT($D$2)*60+($D$2-INT($D$2))*100)</f>
@@ -16984,13 +16982,13 @@
         <v>11.09</v>
       </c>
       <c r="G35" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I35" t="s">
         <v>46</v>
       </c>
       <c r="J35" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K35" t="s">
         <v>92</v>
@@ -17288,13 +17286,13 @@
         <v>11.13</v>
       </c>
       <c r="G41" s="14" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="I41" s="19" t="s">
         <v>81</v>
       </c>
       <c r="J41" s="19" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="K41" s="19" t="s">
         <v>27</v>
@@ -17304,7 +17302,7 @@
         <v>28</v>
       </c>
       <c r="N41" s="19" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="O41">
         <f t="shared" si="7"/>
@@ -17392,13 +17390,13 @@
         <v>11.15</v>
       </c>
       <c r="G43" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I43" t="s">
         <v>46</v>
       </c>
       <c r="J43" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K43" t="s">
         <v>92</v>
@@ -17443,7 +17441,7 @@
         <v>11.15</v>
       </c>
       <c r="F44" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="G44" s="11" t="s">
         <v>32</v>
@@ -17461,7 +17459,7 @@
         <v>35</v>
       </c>
       <c r="N44" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="O44">
         <f t="shared" si="7"/>
@@ -17497,7 +17495,7 @@
         <v>11.16</v>
       </c>
       <c r="F45" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G45" s="11" t="s">
         <v>32</v>
@@ -17515,7 +17513,7 @@
         <v>35</v>
       </c>
       <c r="N45" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="O45">
         <f t="shared" si="7"/>
@@ -17551,7 +17549,7 @@
         <v>11.17</v>
       </c>
       <c r="F46" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="G46" s="11" t="s">
         <v>32</v>
@@ -17569,7 +17567,7 @@
         <v>35</v>
       </c>
       <c r="N46" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="O46">
         <f t="shared" si="7"/>
@@ -17966,7 +17964,7 @@
         <v>11.23</v>
       </c>
       <c r="F54" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="G54" t="s">
         <v>110</v>
@@ -18021,16 +18019,16 @@
         <v>11.23</v>
       </c>
       <c r="F55" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="G55" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I55" t="s">
         <v>46</v>
       </c>
       <c r="J55" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K55" t="s">
         <v>92</v>
@@ -18075,7 +18073,7 @@
         <v>11.24</v>
       </c>
       <c r="F56" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="G56" s="11" t="s">
         <v>32</v>
@@ -18093,7 +18091,7 @@
         <v>35</v>
       </c>
       <c r="N56" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="O56">
         <f t="shared" si="7"/>
@@ -18128,7 +18126,7 @@
         <v>11.25</v>
       </c>
       <c r="F57" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G57" s="11" t="s">
         <v>32</v>
@@ -18146,7 +18144,7 @@
         <v>35</v>
       </c>
       <c r="N57" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="O57">
         <f t="shared" si="7"/>
@@ -18181,7 +18179,7 @@
         <v>11.26</v>
       </c>
       <c r="F58" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G58" s="11" t="s">
         <v>32</v>
@@ -18199,7 +18197,7 @@
         <v>35</v>
       </c>
       <c r="N58" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="O58">
         <f t="shared" si="7"/>
@@ -18235,7 +18233,7 @@
         <v>11.27</v>
       </c>
       <c r="F59" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G59" s="11" t="s">
         <v>32</v>
@@ -18289,7 +18287,7 @@
         <v>11.28</v>
       </c>
       <c r="F60" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="G60" s="11" t="s">
         <v>32</v>
@@ -18344,7 +18342,7 @@
         <v>11.29</v>
       </c>
       <c r="F61" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="G61" t="s">
         <v>69</v>
@@ -18385,7 +18383,7 @@
         <v>11.31</v>
       </c>
       <c r="F62" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="G62" t="s">
         <v>85</v>
@@ -18439,7 +18437,7 @@
         <v>11.32</v>
       </c>
       <c r="F63" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="G63" t="s">
         <v>51</v>
@@ -18493,7 +18491,7 @@
         <v>11.33</v>
       </c>
       <c r="F64" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="G64" s="11" t="s">
         <v>32</v>
@@ -18511,7 +18509,7 @@
         <v>35</v>
       </c>
       <c r="N64" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="O64">
         <f t="shared" si="7"/>
@@ -18546,7 +18544,7 @@
         <v>11.35</v>
       </c>
       <c r="F65" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="G65" s="11" t="s">
         <v>32</v>
@@ -18564,7 +18562,7 @@
         <v>35</v>
       </c>
       <c r="N65" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="O65">
         <f t="shared" si="7"/>
@@ -18600,7 +18598,7 @@
         <v>11.35</v>
       </c>
       <c r="F66" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G66" s="11" t="s">
         <v>32</v>
@@ -18618,7 +18616,7 @@
         <v>35</v>
       </c>
       <c r="N66" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="O66">
         <f t="shared" si="7"/>
@@ -18629,11 +18627,11 @@
         <v>59</v>
       </c>
       <c r="Q66">
-        <f t="shared" ref="Q66:Q97" si="14">P66-O66</f>
+        <f t="shared" ref="Q66:Q67" si="14">P66-O66</f>
         <v>0</v>
       </c>
       <c r="R66" t="str">
-        <f t="shared" ref="R66:R97" si="15">IF(Q66=0,"&lt;1 second","&lt;"&amp;(ROUND(Q66,2)+1)&amp;" seconds")</f>
+        <f t="shared" ref="R66:R67" si="15">IF(Q66=0,"&lt;1 second","&lt;"&amp;(ROUND(Q66,2)+1)&amp;" seconds")</f>
         <v>&lt;1 second</v>
       </c>
       <c r="S66">
@@ -18654,7 +18652,7 @@
         <v>11.36</v>
       </c>
       <c r="F67" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="G67" s="11" t="s">
         <v>32</v>
@@ -18838,13 +18836,13 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>213</v>
+      </c>
+      <c r="B2" t="s">
         <v>214</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>215</v>
-      </c>
-      <c r="C2" t="s">
-        <v>216</v>
       </c>
       <c r="D2" s="3">
         <v>61.28</v>
@@ -18853,7 +18851,7 @@
         <v>61.29</v>
       </c>
       <c r="F2" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="G2" t="s">
         <v>71</v>
@@ -18904,10 +18902,10 @@
         <v>61.3</v>
       </c>
       <c r="F3" t="s">
+        <v>217</v>
+      </c>
+      <c r="G3" s="14" t="s">
         <v>218</v>
-      </c>
-      <c r="G3" s="14" t="s">
-        <v>219</v>
       </c>
       <c r="I3" t="s">
         <v>33</v>
@@ -19057,10 +19055,10 @@
         <v>61.33</v>
       </c>
       <c r="F6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G6" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I6" t="s">
         <v>29</v>
@@ -19108,10 +19106,10 @@
         <v>61.33</v>
       </c>
       <c r="F7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="G7" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I7" t="s">
         <v>29</v>
@@ -19159,7 +19157,7 @@
         <v>61.33</v>
       </c>
       <c r="F8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="G8" t="s">
         <v>51</v>
@@ -19210,7 +19208,7 @@
         <v>61.34</v>
       </c>
       <c r="F9" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G9" t="s">
         <v>109</v>
@@ -19261,10 +19259,10 @@
         <v>61.36</v>
       </c>
       <c r="F10" t="s">
+        <v>217</v>
+      </c>
+      <c r="G10" s="14" t="s">
         <v>218</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>219</v>
       </c>
       <c r="I10" t="s">
         <v>33</v>
@@ -19312,7 +19310,7 @@
         <v>61.38</v>
       </c>
       <c r="F11" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="G11" s="11" t="s">
         <v>32</v>
@@ -19363,10 +19361,10 @@
         <v>61.39</v>
       </c>
       <c r="F12" t="s">
+        <v>223</v>
+      </c>
+      <c r="G12" s="14" t="s">
         <v>224</v>
-      </c>
-      <c r="G12" s="14" t="s">
-        <v>225</v>
       </c>
       <c r="I12" t="s">
         <v>25</v>
@@ -19414,16 +19412,16 @@
         <v>61.41</v>
       </c>
       <c r="F13" t="s">
+        <v>225</v>
+      </c>
+      <c r="G13" s="14" t="s">
         <v>226</v>
       </c>
-      <c r="G13" s="14" t="s">
+      <c r="I13" t="s">
         <v>227</v>
       </c>
-      <c r="I13" t="s">
-        <v>228</v>
-      </c>
       <c r="J13" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="K13" t="s">
         <v>43</v>
@@ -19465,10 +19463,10 @@
         <v>61.42</v>
       </c>
       <c r="F14" t="s">
+        <v>223</v>
+      </c>
+      <c r="G14" s="14" t="s">
         <v>224</v>
-      </c>
-      <c r="G14" s="14" t="s">
-        <v>225</v>
       </c>
       <c r="I14" t="s">
         <v>25</v>
@@ -19515,7 +19513,7 @@
         <v>61.44</v>
       </c>
       <c r="F15" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="G15" t="s">
         <v>85</v>
@@ -19566,16 +19564,16 @@
         <v>61.45</v>
       </c>
       <c r="F16" t="s">
+        <v>225</v>
+      </c>
+      <c r="G16" s="14" t="s">
         <v>226</v>
       </c>
-      <c r="G16" s="14" t="s">
+      <c r="I16" t="s">
         <v>227</v>
       </c>
-      <c r="I16" t="s">
-        <v>228</v>
-      </c>
       <c r="J16" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="K16" t="s">
         <v>43</v>
@@ -19616,7 +19614,7 @@
         <v>61.46</v>
       </c>
       <c r="F17" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="G17" t="s">
         <v>50</v>
@@ -19667,10 +19665,10 @@
         <v>61.46</v>
       </c>
       <c r="F18" t="s">
+        <v>230</v>
+      </c>
+      <c r="G18" s="14" t="s">
         <v>231</v>
-      </c>
-      <c r="G18" s="14" t="s">
-        <v>232</v>
       </c>
       <c r="I18" t="s">
         <v>46</v>
@@ -19718,10 +19716,10 @@
         <v>61.47</v>
       </c>
       <c r="F19" t="s">
+        <v>232</v>
+      </c>
+      <c r="G19" s="14" t="s">
         <v>233</v>
-      </c>
-      <c r="G19" s="14" t="s">
-        <v>234</v>
       </c>
       <c r="I19" t="s">
         <v>46</v>
@@ -19769,16 +19767,16 @@
         <v>61.48</v>
       </c>
       <c r="F20" t="s">
+        <v>234</v>
+      </c>
+      <c r="G20" s="14" t="s">
         <v>235</v>
-      </c>
-      <c r="G20" s="14" t="s">
-        <v>236</v>
       </c>
       <c r="I20" t="s">
         <v>57</v>
       </c>
       <c r="J20" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="K20" t="s">
         <v>27</v>
@@ -19820,10 +19818,10 @@
         <v>61.49</v>
       </c>
       <c r="F21" t="s">
+        <v>237</v>
+      </c>
+      <c r="G21" s="14" t="s">
         <v>238</v>
-      </c>
-      <c r="G21" s="14" t="s">
-        <v>239</v>
       </c>
       <c r="I21" t="s">
         <v>74</v>
@@ -19871,7 +19869,7 @@
         <v>61.49</v>
       </c>
       <c r="F22" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G22" t="s">
         <v>51</v>
@@ -19922,7 +19920,7 @@
         <v>61.5</v>
       </c>
       <c r="F23" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="G23" t="s">
         <v>24</v>
@@ -19973,7 +19971,7 @@
         <v>61.5</v>
       </c>
       <c r="F24" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G24" t="s">
         <v>51</v>
@@ -20023,16 +20021,16 @@
         <v>61.55</v>
       </c>
       <c r="F25" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="G25" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I25" t="s">
         <v>77</v>
       </c>
       <c r="J25" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K25" t="s">
         <v>27</v>
@@ -20073,16 +20071,16 @@
         <v>61.57</v>
       </c>
       <c r="F26" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="G26" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I26" t="s">
         <v>83</v>
       </c>
       <c r="J26" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K26" t="s">
         <v>27</v>
@@ -20123,16 +20121,16 @@
         <v>61.59</v>
       </c>
       <c r="F27" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="G27" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="I27" t="s">
         <v>83</v>
       </c>
       <c r="J27" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="K27" t="s">
         <v>27</v>
@@ -20224,16 +20222,16 @@
         <v>62.06</v>
       </c>
       <c r="F29" t="s">
+        <v>244</v>
+      </c>
+      <c r="G29" s="14" t="s">
         <v>245</v>
-      </c>
-      <c r="G29" s="14" t="s">
-        <v>246</v>
       </c>
       <c r="I29" t="s">
         <v>96</v>
       </c>
       <c r="J29" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="K29" t="s">
         <v>27</v>
@@ -20275,7 +20273,7 @@
         <v>62.06</v>
       </c>
       <c r="F30" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="G30" s="11" t="s">
         <v>32</v>
@@ -20326,7 +20324,7 @@
         <v>62.07</v>
       </c>
       <c r="F31" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="G31" t="s">
         <v>24</v>
@@ -20377,7 +20375,7 @@
         <v>62.08</v>
       </c>
       <c r="F32" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="G32" t="s">
         <v>51</v>
@@ -20427,7 +20425,7 @@
         <v>62.24</v>
       </c>
       <c r="F33" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G33" t="s">
         <v>99</v>
@@ -20517,7 +20515,7 @@
         <v>62.24</v>
       </c>
       <c r="F35" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G35" t="s">
         <v>51</v>
@@ -20568,16 +20566,16 @@
         <v>62.25</v>
       </c>
       <c r="F36" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="G36" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I36" t="s">
         <v>77</v>
       </c>
       <c r="J36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K36" t="s">
         <v>27</v>
@@ -20618,16 +20616,16 @@
         <v>62.28</v>
       </c>
       <c r="F37" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="G37" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I37" t="s">
         <v>77</v>
       </c>
       <c r="J37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K37" t="s">
         <v>27</v>
@@ -20927,13 +20925,13 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>253</v>
+      </c>
+      <c r="C2" t="s">
         <v>254</v>
-      </c>
-      <c r="C2" t="s">
-        <v>255</v>
       </c>
       <c r="D2" s="3">
         <v>24.33</v>
@@ -20943,7 +20941,7 @@
         <v>24.33</v>
       </c>
       <c r="F2" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G2" t="s">
         <v>56</v>
@@ -20994,7 +20992,7 @@
         <v>24.32</v>
       </c>
       <c r="F3" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G3" t="s">
         <v>51</v>
@@ -21044,10 +21042,10 @@
         <v>24.3</v>
       </c>
       <c r="F4" t="s">
+        <v>256</v>
+      </c>
+      <c r="G4" s="14" t="s">
         <v>257</v>
-      </c>
-      <c r="G4" s="14" t="s">
-        <v>258</v>
       </c>
       <c r="I4" s="19" t="s">
         <v>115</v>
@@ -21095,7 +21093,7 @@
         <v>24.29</v>
       </c>
       <c r="F5" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G5" t="s">
         <v>45</v>
@@ -21145,7 +21143,7 @@
         <v>24.27</v>
       </c>
       <c r="F6" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="G6" t="s">
         <v>56</v>
@@ -21196,7 +21194,7 @@
         <v>24.27</v>
       </c>
       <c r="F7" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="G7" t="s">
         <v>45</v>
@@ -21247,7 +21245,7 @@
         <v>24.26</v>
       </c>
       <c r="F8" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="G8" s="11" t="s">
         <v>32</v>
@@ -21298,7 +21296,7 @@
         <v>24.26</v>
       </c>
       <c r="F9" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="G9" s="11" t="s">
         <v>32</v>
@@ -21348,10 +21346,10 @@
         <v>24.23</v>
       </c>
       <c r="F10" t="s">
+        <v>261</v>
+      </c>
+      <c r="G10" s="14" t="s">
         <v>262</v>
-      </c>
-      <c r="G10" s="14" t="s">
-        <v>263</v>
       </c>
       <c r="I10" t="s">
         <v>33</v>
@@ -21399,10 +21397,10 @@
         <v>24.22</v>
       </c>
       <c r="F11" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="G11" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I11" t="s">
         <v>46</v>
@@ -21450,16 +21448,16 @@
         <v>24.21</v>
       </c>
       <c r="F12" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G12" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="I12" t="s">
         <v>81</v>
       </c>
       <c r="J12" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="K12" t="s">
         <v>43</v>
@@ -21501,7 +21499,7 @@
         <v>24.2</v>
       </c>
       <c r="F13" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="G13" t="s">
         <v>109</v>
@@ -21552,7 +21550,7 @@
         <v>24.17</v>
       </c>
       <c r="F14" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="G14" t="s">
         <v>85</v>
@@ -21654,7 +21652,7 @@
         <v>24.16</v>
       </c>
       <c r="F16" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G16" t="s">
         <v>51</v>
@@ -21705,10 +21703,10 @@
         <v>24.15</v>
       </c>
       <c r="F17" t="s">
+        <v>265</v>
+      </c>
+      <c r="G17" s="14" t="s">
         <v>266</v>
-      </c>
-      <c r="G17" s="14" t="s">
-        <v>267</v>
       </c>
       <c r="I17" s="19" t="s">
         <v>77</v>
@@ -21755,10 +21753,10 @@
         <v>24.14</v>
       </c>
       <c r="F18" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G18" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I18" t="s">
         <v>46</v>
@@ -21805,10 +21803,10 @@
         <v>24.13</v>
       </c>
       <c r="F19" t="s">
+        <v>268</v>
+      </c>
+      <c r="G19" s="14" t="s">
         <v>269</v>
-      </c>
-      <c r="G19" s="14" t="s">
-        <v>270</v>
       </c>
       <c r="I19" t="s">
         <v>77</v>
@@ -21856,10 +21854,10 @@
         <v>24.12</v>
       </c>
       <c r="F20" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="G20" s="14" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I20" s="19" t="s">
         <v>77</v>
@@ -21907,10 +21905,10 @@
         <v>24.12</v>
       </c>
       <c r="F21" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="G21" s="14" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I21" t="s">
         <v>77</v>
@@ -21958,7 +21956,7 @@
         <v>24.11</v>
       </c>
       <c r="F22" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="G22" t="s">
         <v>45</v>
@@ -22009,16 +22007,16 @@
         <v>24.1</v>
       </c>
       <c r="F23" t="s">
+        <v>273</v>
+      </c>
+      <c r="G23" s="14" t="s">
         <v>274</v>
-      </c>
-      <c r="G23" s="14" t="s">
-        <v>275</v>
       </c>
       <c r="I23" s="19" t="s">
         <v>83</v>
       </c>
       <c r="J23" s="19" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="K23" t="s">
         <v>27</v>
@@ -22111,7 +22109,7 @@
         <v>24.09</v>
       </c>
       <c r="F25" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G25" t="s">
         <v>51</v>
@@ -22161,10 +22159,10 @@
         <v>24.08</v>
       </c>
       <c r="F26" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="G26" s="14" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I26" s="19" t="s">
         <v>77</v>
@@ -22212,10 +22210,10 @@
         <v>24.07</v>
       </c>
       <c r="F27" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="G27" s="14" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I27" t="s">
         <v>77</v>
@@ -22262,7 +22260,7 @@
         <v>24.05</v>
       </c>
       <c r="F28" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="G28" s="11" t="s">
         <v>32</v>
@@ -22414,16 +22412,16 @@
         <v>23.56</v>
       </c>
       <c r="F31" t="s">
+        <v>279</v>
+      </c>
+      <c r="G31" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="G31" s="14" t="s">
+      <c r="I31" t="s">
         <v>281</v>
       </c>
-      <c r="I31" t="s">
-        <v>282</v>
-      </c>
       <c r="J31" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="K31" t="s">
         <v>27</v>
@@ -22516,7 +22514,7 @@
         <v>23.55</v>
       </c>
       <c r="F33" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="O33">
         <f t="shared" si="0"/>
@@ -22551,16 +22549,16 @@
         <v>23.54</v>
       </c>
       <c r="F34" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="G34" s="14" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="I34" t="s">
         <v>77</v>
       </c>
       <c r="J34" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K34" t="s">
         <v>27</v>
@@ -22602,16 +22600,16 @@
         <v>23.53</v>
       </c>
       <c r="F35" t="s">
+        <v>279</v>
+      </c>
+      <c r="G35" s="14" t="s">
         <v>280</v>
       </c>
-      <c r="G35" s="14" t="s">
+      <c r="I35" t="s">
         <v>281</v>
       </c>
-      <c r="I35" t="s">
-        <v>282</v>
-      </c>
       <c r="J35" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="K35" t="s">
         <v>43</v>
@@ -22652,7 +22650,7 @@
         <v>23.5</v>
       </c>
       <c r="F36" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="G36" t="s">
         <v>121</v>
@@ -22702,10 +22700,10 @@
         <v>23.47</v>
       </c>
       <c r="F37" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="G37" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="I37" t="s">
         <v>46</v>
@@ -22753,7 +22751,7 @@
         <v>23.45</v>
       </c>
       <c r="F38" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="G38" s="11" t="s">
         <v>32</v>
@@ -22855,7 +22853,7 @@
         <v>23.44</v>
       </c>
       <c r="F40" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G40" t="s">
         <v>51</v>
@@ -22906,16 +22904,16 @@
         <v>23.44</v>
       </c>
       <c r="F41" t="s">
+        <v>286</v>
+      </c>
+      <c r="G41" s="14" t="s">
         <v>287</v>
-      </c>
-      <c r="G41" s="14" t="s">
-        <v>288</v>
       </c>
       <c r="I41" s="19" t="s">
         <v>77</v>
       </c>
       <c r="J41" s="19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="K41" t="s">
         <v>27</v>
@@ -22956,7 +22954,7 @@
         <v>23.4</v>
       </c>
       <c r="F42" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G42" t="s">
         <v>121</v>
@@ -23007,7 +23005,7 @@
         <v>23.32</v>
       </c>
       <c r="F43" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="G43" s="11" t="s">
         <v>32</v>
@@ -23058,7 +23056,7 @@
         <v>23.28</v>
       </c>
       <c r="F44" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="G44" t="s">
         <v>121</v>
@@ -23101,226 +23099,115 @@
       </c>
     </row>
     <row r="45" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="E45" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E45" s="3"/>
     </row>
     <row r="46" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="E46" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E46" s="3"/>
     </row>
     <row r="47" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="E47" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E47" s="3"/>
     </row>
     <row r="48" spans="4:20" x14ac:dyDescent="0.2">
-      <c r="E48" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E48" s="3"/>
     </row>
     <row r="49" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E49" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E49" s="3"/>
     </row>
     <row r="50" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E50" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E50" s="3"/>
     </row>
     <row r="51" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E51" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E51" s="3"/>
     </row>
     <row r="52" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E52" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E52" s="3"/>
     </row>
     <row r="53" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E53" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E53" s="3"/>
     </row>
     <row r="54" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E54" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E54" s="3"/>
     </row>
     <row r="55" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E55" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E55" s="3"/>
     </row>
     <row r="56" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E56" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E56" s="3"/>
     </row>
     <row r="57" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E57" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E57" s="3"/>
     </row>
     <row r="58" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E58" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E58" s="3"/>
     </row>
     <row r="59" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E59" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E59" s="3"/>
     </row>
     <row r="60" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E60" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E60" s="3"/>
     </row>
     <row r="61" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E61" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E61" s="3"/>
     </row>
     <row r="62" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E62" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E62" s="3"/>
     </row>
     <row r="63" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E63" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E63" s="3"/>
     </row>
     <row r="64" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E64" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E64" s="3"/>
     </row>
     <row r="65" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E65" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E65" s="3"/>
     </row>
     <row r="66" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E66" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E66" s="3"/>
     </row>
     <row r="67" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E67" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E67" s="3"/>
     </row>
     <row r="68" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E68" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E68" s="3"/>
     </row>
     <row r="69" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E69" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E69" s="3"/>
     </row>
     <row r="70" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E70" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E70" s="3"/>
     </row>
     <row r="71" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E71" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E71" s="3"/>
     </row>
     <row r="72" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E72" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E72" s="3"/>
     </row>
     <row r="73" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E73" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E73" s="3"/>
     </row>
     <row r="74" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E74" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E74" s="3"/>
     </row>
     <row r="75" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E75" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E75" s="3"/>
     </row>
     <row r="76" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E76" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E76" s="3"/>
     </row>
     <row r="77" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E77" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E77" s="3"/>
     </row>
     <row r="78" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E78" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E78" s="3"/>
     </row>
     <row r="79" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E79" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E79" s="3"/>
     </row>
     <row r="80" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E80" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E80" s="3"/>
     </row>
     <row r="81" spans="5:5" x14ac:dyDescent="0.2">
-      <c r="E81" s="3">
-        <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
+      <c r="E81" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="3">
@@ -23461,13 +23348,13 @@
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
+        <v>290</v>
+      </c>
+      <c r="B2" s="10" t="s">
         <v>291</v>
       </c>
-      <c r="B2" s="10" t="s">
+      <c r="C2" t="s">
         <v>292</v>
-      </c>
-      <c r="C2" t="s">
-        <v>293</v>
       </c>
       <c r="D2" s="3">
         <v>94.02</v>
@@ -23477,7 +23364,7 @@
         <v>94.02</v>
       </c>
       <c r="F2" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="G2" t="s">
         <v>51</v>
@@ -23528,7 +23415,7 @@
         <v>94.02</v>
       </c>
       <c r="F3" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="G3" t="s">
         <v>24</v>
@@ -23579,7 +23466,7 @@
         <v>94.03</v>
       </c>
       <c r="F4" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="G4" t="s">
         <v>45</v>
@@ -23629,7 +23516,7 @@
         <v>94.05</v>
       </c>
       <c r="F5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="G5" t="s">
         <v>90</v>
@@ -23679,16 +23566,16 @@
         <v>94.1</v>
       </c>
       <c r="F6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I6" t="s">
         <v>46</v>
       </c>
       <c r="J6" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K6" t="s">
         <v>92</v>
@@ -23730,7 +23617,7 @@
         <v>94.11</v>
       </c>
       <c r="F7" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="G7" t="s">
         <v>117</v>
@@ -23781,16 +23668,16 @@
         <v>94.13</v>
       </c>
       <c r="F8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="G8" t="s">
+        <v>226</v>
+      </c>
+      <c r="I8" t="s">
         <v>227</v>
       </c>
-      <c r="I8" t="s">
-        <v>228</v>
-      </c>
       <c r="J8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="K8" t="s">
         <v>43</v>
@@ -23832,7 +23719,7 @@
         <v>94.15</v>
       </c>
       <c r="F9" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="G9" t="s">
         <v>32</v>
@@ -23883,7 +23770,7 @@
         <v>94.16</v>
       </c>
       <c r="F10" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="G10" t="s">
         <v>32</v>
@@ -23934,16 +23821,16 @@
         <v>94.17</v>
       </c>
       <c r="F11" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="I11" t="s">
         <v>57</v>
       </c>
       <c r="J11" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="K11" t="s">
         <v>27</v>
@@ -23984,7 +23871,7 @@
         <v>94.21</v>
       </c>
       <c r="F12" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="G12" t="s">
         <v>82</v>
@@ -24034,7 +23921,7 @@
         <v>94.23</v>
       </c>
       <c r="F13" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="G13" t="s">
         <v>32</v>
@@ -24085,7 +23972,7 @@
         <v>94.25</v>
       </c>
       <c r="F14" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G14" t="s">
         <v>45</v>
@@ -24135,7 +24022,7 @@
         <v>94.28</v>
       </c>
       <c r="F15" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G15" t="s">
         <v>85</v>
@@ -24185,10 +24072,10 @@
         <v>94.29</v>
       </c>
       <c r="F16" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G16" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I16" s="19" t="s">
         <v>77</v>
@@ -24236,10 +24123,10 @@
         <v>94.3</v>
       </c>
       <c r="F17" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G17" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I17" s="19" t="s">
         <v>77</v>
@@ -24288,7 +24175,7 @@
         <v>94.3</v>
       </c>
       <c r="G18" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I18" s="19" t="s">
         <v>77</v>
@@ -24337,7 +24224,7 @@
         <v>94.3</v>
       </c>
       <c r="G19" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I19" s="19" t="s">
         <v>77</v>
@@ -24385,7 +24272,7 @@
         <v>94.32</v>
       </c>
       <c r="G20" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I20" s="19" t="s">
         <v>77</v>
@@ -24433,7 +24320,7 @@
         <v>94.33</v>
       </c>
       <c r="G21" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I21" s="19" t="s">
         <v>77</v>
@@ -24481,7 +24368,7 @@
         <v>94.34</v>
       </c>
       <c r="G22" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I22" s="19" t="s">
         <v>77</v>
@@ -24529,7 +24416,7 @@
         <v>94.35</v>
       </c>
       <c r="G23" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I23" s="19" t="s">
         <v>77</v>
@@ -24577,7 +24464,7 @@
         <v>94.37</v>
       </c>
       <c r="G24" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="I24" s="19" t="s">
         <v>77</v>
@@ -24720,7 +24607,7 @@
         <v>94.45</v>
       </c>
       <c r="F27" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="G27" t="s">
         <v>51</v>
@@ -24771,10 +24658,10 @@
         <v>94.45</v>
       </c>
       <c r="F28" t="s">
+        <v>308</v>
+      </c>
+      <c r="G28" s="15" t="s">
         <v>309</v>
-      </c>
-      <c r="G28" s="15" t="s">
-        <v>310</v>
       </c>
       <c r="I28" s="19" t="s">
         <v>25</v>
@@ -24823,7 +24710,7 @@
         <v>94.48</v>
       </c>
       <c r="G29" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="I29" t="s">
         <v>81</v>
@@ -24870,7 +24757,7 @@
         <v>94.5</v>
       </c>
       <c r="F30" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="G30" t="s">
         <v>32</v>
@@ -24920,10 +24807,10 @@
         <v>94.52</v>
       </c>
       <c r="F31" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="G31" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="I31" t="s">
         <v>115</v>
@@ -24971,7 +24858,7 @@
         <v>94.53</v>
       </c>
       <c r="F32" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G32" t="s">
         <v>32</v>
@@ -25021,16 +24908,16 @@
         <v>94.57</v>
       </c>
       <c r="F33" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="G33" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I33" t="s">
         <v>46</v>
       </c>
       <c r="J33" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K33" t="s">
         <v>92</v>
@@ -25120,7 +25007,7 @@
         <v>94.58</v>
       </c>
       <c r="G35" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I35" t="s">
         <v>29</v>
@@ -25524,10 +25411,10 @@
         <v>21</v>
       </c>
       <c r="B2" s="10" t="s">
+        <v>315</v>
+      </c>
+      <c r="C2" t="s">
         <v>316</v>
-      </c>
-      <c r="C2" t="s">
-        <v>317</v>
       </c>
       <c r="D2" s="3">
         <v>14.57</v>
@@ -25536,7 +25423,7 @@
         <v>14.59</v>
       </c>
       <c r="F2" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="G2" t="s">
         <v>121</v>
@@ -25586,16 +25473,16 @@
         <v>14.59</v>
       </c>
       <c r="F3" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="G3" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I3" t="s">
         <v>46</v>
       </c>
       <c r="J3" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K3" t="s">
         <v>92</v>
@@ -25636,7 +25523,7 @@
         <v>15.01</v>
       </c>
       <c r="F4" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="G4" t="s">
         <v>32</v>
@@ -25784,7 +25671,7 @@
         <v>15.14</v>
       </c>
       <c r="F7" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="G7" t="s">
         <v>32</v>
@@ -25835,17 +25722,17 @@
         <v>15.14</v>
       </c>
       <c r="F8" t="s">
+        <v>321</v>
+      </c>
+      <c r="G8" s="19" t="s">
         <v>322</v>
-      </c>
-      <c r="G8" s="19" t="s">
-        <v>323</v>
       </c>
       <c r="H8" s="19"/>
       <c r="I8" s="19" t="s">
         <v>57</v>
       </c>
       <c r="J8" s="19" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="K8" s="19" t="s">
         <v>27</v>
@@ -25887,7 +25774,7 @@
         <v>15.16</v>
       </c>
       <c r="F9" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="G9" t="s">
         <v>76</v>
@@ -25937,7 +25824,7 @@
         <v>15.27</v>
       </c>
       <c r="F10" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="G10" t="s">
         <v>32</v>
@@ -25988,17 +25875,17 @@
         <v>15.27</v>
       </c>
       <c r="F11" t="s">
+        <v>321</v>
+      </c>
+      <c r="G11" s="19" t="s">
         <v>322</v>
-      </c>
-      <c r="G11" s="19" t="s">
-        <v>323</v>
       </c>
       <c r="H11" s="19"/>
       <c r="I11" s="19" t="s">
         <v>57</v>
       </c>
       <c r="J11" s="19" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="K11" s="19" t="s">
         <v>27</v>
@@ -26040,7 +25927,7 @@
         <v>15.29</v>
       </c>
       <c r="G12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="I12" t="s">
         <v>77</v>
@@ -26135,14 +26022,14 @@
         <v>15.35</v>
       </c>
       <c r="G14" s="19" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="H14" s="19"/>
       <c r="I14" s="19" t="s">
         <v>57</v>
       </c>
       <c r="J14" s="19" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="K14" s="19" t="s">
         <v>27</v>
@@ -26328,7 +26215,7 @@
         <v>15.4</v>
       </c>
       <c r="F18" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="G18" t="s">
         <v>32</v>
@@ -26378,7 +26265,7 @@
         <v>15.44</v>
       </c>
       <c r="F19" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="G19" t="s">
         <v>32</v>
@@ -26429,7 +26316,7 @@
         <v>15.44</v>
       </c>
       <c r="G20" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I20" t="s">
         <v>115</v>
@@ -26477,7 +26364,7 @@
         <v>15.45</v>
       </c>
       <c r="F21" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G21" t="s">
         <v>32</v>
@@ -26624,7 +26511,7 @@
         <v>15.46</v>
       </c>
       <c r="G24" s="17" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="I24" t="s">
         <v>74</v>
@@ -26719,7 +26606,7 @@
         <v>15.47</v>
       </c>
       <c r="F26" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="G26" t="s">
         <v>32</v>
@@ -26769,13 +26656,13 @@
         <v>15.48</v>
       </c>
       <c r="G27" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="I27" t="s">
         <v>46</v>
       </c>
       <c r="J27" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K27" t="s">
         <v>92</v>
@@ -26816,7 +26703,7 @@
         <v>15.49</v>
       </c>
       <c r="F28" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="G28" t="s">
         <v>45</v>
@@ -26915,16 +26802,16 @@
         <v>15.49</v>
       </c>
       <c r="F30" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="G30" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="I30" t="s">
         <v>46</v>
       </c>
       <c r="J30" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K30" t="s">
         <v>92</v>
@@ -27062,7 +26949,7 @@
         <v>15.51</v>
       </c>
       <c r="G33" s="17" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="I33" t="s">
         <v>74</v>
@@ -27158,13 +27045,13 @@
         <v>15.53</v>
       </c>
       <c r="G35" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="I35" t="s">
         <v>46</v>
       </c>
       <c r="J35" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="K35" t="s">
         <v>92</v>
@@ -27205,13 +27092,13 @@
         <v>15.54</v>
       </c>
       <c r="G36" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I36" t="s">
         <v>46</v>
       </c>
       <c r="J36" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K36" t="s">
         <v>92</v>
@@ -27299,13 +27186,13 @@
         <v>15.55</v>
       </c>
       <c r="G38" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I38" t="s">
         <v>46</v>
       </c>
       <c r="J38" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K38" t="s">
         <v>92</v>
@@ -27346,13 +27233,13 @@
         <v>15.56</v>
       </c>
       <c r="G39" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="I39" t="s">
         <v>46</v>
       </c>
       <c r="J39" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="K39" t="s">
         <v>92</v>
@@ -27753,7 +27640,7 @@
         <v>86.58</v>
       </c>
       <c r="G3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I3" t="s">
         <v>29</v>
@@ -27906,7 +27793,7 @@
         <v>40</v>
       </c>
       <c r="G6" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I6" t="s">
         <v>29</v>
@@ -28053,7 +27940,7 @@
         <v>87.04</v>
       </c>
       <c r="G9" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I9" t="s">
         <v>29</v>
@@ -28397,7 +28284,7 @@
         <v>87.14</v>
       </c>
       <c r="G16" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I16" t="s">
         <v>29</v>
@@ -28883,7 +28770,7 @@
         <v>40</v>
       </c>
       <c r="G26" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I26" t="s">
         <v>29</v>
@@ -28982,7 +28869,7 @@
         <v>40</v>
       </c>
       <c r="G28" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I28" t="s">
         <v>29</v>
@@ -29180,7 +29067,7 @@
         <v>87.26</v>
       </c>
       <c r="G32" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I32" t="s">
         <v>29</v>
@@ -29305,11 +29192,11 @@
         <v>35</v>
       </c>
       <c r="Q34">
-        <f t="shared" ref="Q34:Q65" si="11">P34-O34</f>
+        <f t="shared" ref="Q34:Q58" si="11">P34-O34</f>
         <v>0</v>
       </c>
       <c r="R34" t="str">
-        <f t="shared" ref="R34:R65" si="12">IF(Q34=0,"&lt;1 second","&lt;"&amp;(ROUND(Q34,2)+1)&amp;" seconds")</f>
+        <f t="shared" ref="R34:R58" si="12">IF(Q34=0,"&lt;1 second","&lt;"&amp;(ROUND(Q34,2)+1)&amp;" seconds")</f>
         <v>&lt;1 second</v>
       </c>
       <c r="S34">
@@ -29380,7 +29267,7 @@
         <v>40</v>
       </c>
       <c r="G36" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I36" t="s">
         <v>29</v>
@@ -30148,7 +30035,7 @@
         <v>75</v>
       </c>
       <c r="G52" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="I52" t="s">
         <v>29</v>

</xml_diff>